<commit_message>
design analysis data added
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY COMPUTER\Yogi\Sem 6\CE6030\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0ADFF9-EDA7-4F27-B669-4D57261B286F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE5B651-8D2A-42A7-A895-681CC9DFB313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Bus</t>
   </si>
@@ -76,19 +76,65 @@
   </si>
   <si>
     <t>For calculation of VDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LDF = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">VDF = </t>
+  </si>
+  <si>
+    <t xml:space="preserve">n (Design life in years) </t>
+  </si>
+  <si>
+    <t>r (rate of traffic growth)</t>
+  </si>
+  <si>
+    <t>Mix design parameters of bituminous layer: 3% air voids and 11.5% effective bitumen content</t>
+  </si>
+  <si>
+    <t>Effective CBR of the subgrade = 9 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (for three lane in each direction)</t>
+  </si>
+  <si>
+    <t>% composition</t>
+  </si>
+  <si>
+    <t>Truck- 2-axle trucks, MAV- Multi-axle (more than two axles) trucks, LCVs – Light Commercial Vehicles.</t>
+  </si>
+  <si>
+    <t>Period - Feb, 2016</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -105,7 +151,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -162,22 +208,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -455,7 +519,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:J17"/>
+  <dimension ref="B2:J26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
@@ -481,35 +545,41 @@
       <c r="B4" t="s">
         <v>8</v>
       </c>
+      <c r="E4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="J5" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B6" s="2">
+      <c r="B6" s="1">
         <v>42401</v>
       </c>
       <c r="C6">
@@ -532,8 +602,8 @@
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B7" s="2">
-        <f>B6+3</f>
+      <c r="B7" s="1">
+        <f t="shared" ref="B7:B15" si="0">B6+3</f>
         <v>42404</v>
       </c>
       <c r="C7">
@@ -556,8 +626,8 @@
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B8" s="2">
-        <f>B7+3</f>
+      <c r="B8" s="1">
+        <f t="shared" si="0"/>
         <v>42407</v>
       </c>
       <c r="C8">
@@ -580,8 +650,8 @@
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B9" s="2">
-        <f>B8+3</f>
+      <c r="B9" s="1">
+        <f t="shared" si="0"/>
         <v>42410</v>
       </c>
       <c r="C9">
@@ -604,8 +674,8 @@
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="2">
-        <f>B9+3</f>
+      <c r="B10" s="1">
+        <f t="shared" si="0"/>
         <v>42413</v>
       </c>
       <c r="C10">
@@ -628,8 +698,8 @@
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B11" s="2">
-        <f>B10+3</f>
+      <c r="B11" s="1">
+        <f t="shared" si="0"/>
         <v>42416</v>
       </c>
       <c r="C11">
@@ -652,8 +722,8 @@
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B12" s="2">
-        <f>B11+3</f>
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
         <v>42419</v>
       </c>
       <c r="C12">
@@ -676,8 +746,8 @@
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B13" s="2">
-        <f>B12+3</f>
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
         <v>42422</v>
       </c>
       <c r="C13">
@@ -700,8 +770,8 @@
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B14" s="2">
-        <f>B13+3</f>
+      <c r="B14" s="1">
+        <f t="shared" si="0"/>
         <v>42425</v>
       </c>
       <c r="C14">
@@ -724,8 +794,8 @@
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B15" s="2">
-        <f>B14+3</f>
+      <c r="B15" s="1">
+        <f t="shared" si="0"/>
         <v>42428</v>
       </c>
       <c r="C15">
@@ -748,36 +818,104 @@
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <f>AVERAGE(C6:C15)</f>
         <v>9053.1</v>
       </c>
-      <c r="D16" s="6">
-        <f t="shared" ref="D16:H16" si="0">AVERAGE(D6:D15)</f>
+      <c r="D16" s="5">
+        <f t="shared" ref="D16:H16" si="1">AVERAGE(D6:D15)</f>
         <v>829.1</v>
       </c>
-      <c r="E16" s="6">
-        <f t="shared" si="0"/>
+      <c r="E16" s="5">
+        <f t="shared" si="1"/>
         <v>613</v>
       </c>
-      <c r="F16" s="6">
-        <f t="shared" si="0"/>
+      <c r="F16" s="5">
+        <f t="shared" si="1"/>
         <v>1435</v>
       </c>
-      <c r="G16" s="6">
-        <f t="shared" si="0"/>
+      <c r="G16" s="5">
+        <f t="shared" si="1"/>
         <v>454.9</v>
       </c>
-      <c r="H16" s="6">
-        <f t="shared" si="0"/>
+      <c r="H16" s="5">
+        <f t="shared" si="1"/>
         <v>446.1</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="1"/>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B17" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="12">
+        <f>C16/(SUM($C$16:$H$16))</f>
+        <v>0.70555365047696239</v>
+      </c>
+      <c r="D17" s="11">
+        <f t="shared" ref="D17:H17" si="2">D16/(SUM($C$16:$H$16))</f>
+        <v>6.4615936155620668E-2</v>
+      </c>
+      <c r="E17" s="11">
+        <f t="shared" si="2"/>
+        <v>4.7774175447347092E-2</v>
+      </c>
+      <c r="F17" s="11">
+        <f t="shared" si="2"/>
+        <v>0.11183677286613879</v>
+      </c>
+      <c r="G17" s="11">
+        <f t="shared" si="2"/>
+        <v>3.5452646673732775E-2</v>
+      </c>
+      <c r="H17" s="11">
+        <f t="shared" si="2"/>
+        <v>3.4766818380198267E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="D22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B23" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="7">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Rigid pavement pdf added
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MY COMPUTER\Yogi\Sem 6\CE6030\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7FB2EF0-04A9-45C4-B25B-E371EB3E1525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E744E5A4-00A3-49DA-B5D6-C71A9D009EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Flexible Pavement Design" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="105">
   <si>
     <t>Bus</t>
   </si>
@@ -406,6 +406,27 @@
   <si>
     <t>Effective bitumen content</t>
   </si>
+  <si>
+    <t>Initial construction cost</t>
+  </si>
+  <si>
+    <t>Routine maintenance cost</t>
+  </si>
+  <si>
+    <t>Periodic maintenance cost</t>
+  </si>
+  <si>
+    <t>Rehabiliation cost</t>
+  </si>
+  <si>
+    <t>Salvage value</t>
+  </si>
+  <si>
+    <t>Fuel cost</t>
+  </si>
+  <si>
+    <t>Time saving benefits</t>
+  </si>
 </sst>
 </file>
 
@@ -414,11 +435,11 @@
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
-    <numFmt numFmtId="171" formatCode="0.000"/>
-    <numFmt numFmtId="179" formatCode="0.000E+00"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.000E+00"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -511,6 +532,14 @@
       <name val="Calibri Light"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -736,7 +765,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -794,17 +823,77 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -818,70 +907,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1896,93 +1923,93 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="63"/>
+      <c r="E6" s="63"/>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="63"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="27" t="s">
+      <c r="C7" s="60" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="29"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="62"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="29"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
+      <c r="G8" s="61"/>
+      <c r="H8" s="62"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="60" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="29"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="61"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="62"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="60" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="29"/>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="61"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="62"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="29"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="62"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="62"/>
     </row>
     <row r="15" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="6" t="s">
@@ -2306,52 +2333,52 @@
       </c>
     </row>
     <row r="30" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B30" s="42" t="s">
+      <c r="B30" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="C30" s="42"/>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="42"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="42"/>
-      <c r="J30" s="42"/>
-      <c r="K30" s="42"/>
-      <c r="L30" s="42"/>
-      <c r="M30" s="42"/>
-      <c r="N30" s="42"/>
-      <c r="O30" s="42"/>
-      <c r="P30" s="42"/>
-      <c r="Q30" s="42"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
+      <c r="G30" s="56"/>
+      <c r="H30" s="56"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="56"/>
+      <c r="K30" s="56"/>
+      <c r="L30" s="56"/>
+      <c r="M30" s="56"/>
+      <c r="N30" s="56"/>
+      <c r="O30" s="56"/>
+      <c r="P30" s="56"/>
+      <c r="Q30" s="56"/>
     </row>
     <row r="32" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B32" s="24"/>
-      <c r="C32" s="44" t="s">
+      <c r="C32" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="D32" s="44"/>
-      <c r="E32" s="44" t="s">
+      <c r="D32" s="59"/>
+      <c r="E32" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44" t="s">
+      <c r="F32" s="59"/>
+      <c r="G32" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44" t="s">
+      <c r="H32" s="59"/>
+      <c r="I32" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="J32" s="44"/>
-      <c r="K32" s="44" t="s">
+      <c r="J32" s="59"/>
+      <c r="K32" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="L32" s="44"/>
-      <c r="M32" s="44" t="s">
+      <c r="L32" s="59"/>
+      <c r="M32" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="N32" s="44"/>
-      <c r="P32" s="41" t="s">
+      <c r="N32" s="59"/>
+      <c r="P32" s="28" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2359,30 +2386,30 @@
       <c r="B33" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C33" s="44">
+      <c r="C33" s="59">
         <v>1700</v>
       </c>
-      <c r="D33" s="44"/>
-      <c r="E33" s="44">
+      <c r="D33" s="59"/>
+      <c r="E33" s="59">
         <v>10000</v>
       </c>
-      <c r="F33" s="44"/>
-      <c r="G33" s="44">
+      <c r="F33" s="59"/>
+      <c r="G33" s="59">
         <v>18500</v>
       </c>
-      <c r="H33" s="44"/>
-      <c r="I33" s="44">
+      <c r="H33" s="59"/>
+      <c r="I33" s="59">
         <v>5000</v>
       </c>
-      <c r="J33" s="44"/>
-      <c r="K33" s="44">
+      <c r="J33" s="59"/>
+      <c r="K33" s="59">
         <v>45500</v>
       </c>
-      <c r="L33" s="44"/>
-      <c r="M33" s="44">
+      <c r="L33" s="59"/>
+      <c r="M33" s="59">
         <v>28000</v>
       </c>
-      <c r="N33" s="44"/>
+      <c r="N33" s="59"/>
       <c r="P33" t="s">
         <v>50</v>
       </c>
@@ -2432,51 +2459,51 @@
       <c r="B35" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="46">
+      <c r="C35" s="30">
         <f>$C$33/2</f>
         <v>850</v>
       </c>
-      <c r="D35" s="46">
+      <c r="D35" s="30">
         <f>$C$33/2</f>
         <v>850</v>
       </c>
-      <c r="E35" s="46">
+      <c r="E35" s="30">
         <f>$E$33/3</f>
         <v>3333.3333333333335</v>
       </c>
-      <c r="F35" s="46">
+      <c r="F35" s="30">
         <f>$E$33*2/3</f>
         <v>6666.666666666667</v>
       </c>
-      <c r="G35" s="46">
+      <c r="G35" s="30">
         <f>$G$33/5</f>
         <v>3700</v>
       </c>
-      <c r="H35" s="46">
+      <c r="H35" s="30">
         <f>$G$33*4/5</f>
         <v>14800</v>
       </c>
-      <c r="I35" s="46">
+      <c r="I35" s="30">
         <f>$I$33/2</f>
         <v>2500</v>
       </c>
-      <c r="J35" s="46">
+      <c r="J35" s="30">
         <f>$I$33/2</f>
         <v>2500</v>
       </c>
-      <c r="K35" s="46">
+      <c r="K35" s="30">
         <f>$K$33*2/5</f>
         <v>18200</v>
       </c>
-      <c r="L35" s="46">
+      <c r="L35" s="30">
         <f>$K$33*3/5</f>
         <v>27300</v>
       </c>
-      <c r="M35" s="46">
+      <c r="M35" s="30">
         <f>$M$33/4</f>
         <v>7000</v>
       </c>
-      <c r="N35" s="46">
+      <c r="N35" s="30">
         <f>$M$33*3/4</f>
         <v>21000</v>
       </c>
@@ -2488,51 +2515,51 @@
       <c r="B36" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C36" s="49">
+      <c r="C36" s="41">
         <f>(C35*10/1000/65)^4</f>
         <v>2.9243023703651833E-4</v>
       </c>
-      <c r="D36" s="49">
+      <c r="D36" s="41">
         <f>(D35*10/1000/65)^4</f>
         <v>2.9243023703651833E-4</v>
       </c>
-      <c r="E36" s="49">
-        <f t="shared" ref="E36:N36" si="3">(E35*10/1000/65)^4</f>
+      <c r="E36" s="41">
+        <f t="shared" ref="E36:M36" si="3">(E35*10/1000/65)^4</f>
         <v>6.9161046251017447E-2</v>
       </c>
-      <c r="F36" s="49">
+      <c r="F36" s="41">
         <f>(F35*10/1000/80)^4</f>
         <v>0.48225308641975323</v>
       </c>
-      <c r="G36" s="49">
+      <c r="G36" s="41">
         <f t="shared" si="3"/>
         <v>0.10499133783831098</v>
       </c>
-      <c r="H36" s="49">
+      <c r="H36" s="41">
         <f>(H35*10/1000/148)^4</f>
         <v>1</v>
       </c>
-      <c r="I36" s="49">
+      <c r="I36" s="41">
         <f t="shared" si="3"/>
         <v>2.1882987290360985E-2</v>
       </c>
-      <c r="J36" s="49">
+      <c r="J36" s="41">
         <f t="shared" si="3"/>
         <v>2.1882987290360985E-2</v>
       </c>
-      <c r="K36" s="49">
+      <c r="K36" s="41">
         <f t="shared" si="3"/>
         <v>61.465599999999981</v>
       </c>
-      <c r="L36" s="49">
+      <c r="L36" s="41">
         <f>(L35*10/1000/224)^4</f>
         <v>2.2062692642211914</v>
       </c>
-      <c r="M36" s="49">
+      <c r="M36" s="41">
         <f t="shared" si="3"/>
         <v>1.3450509435944118</v>
       </c>
-      <c r="N36" s="49">
+      <c r="N36" s="41">
         <f>(N35*10/1000/148)^4</f>
         <v>4.0535013067180454</v>
       </c>
@@ -2541,171 +2568,170 @@
       <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C37" s="50">
+      <c r="C37" s="57">
         <f>C36+D36</f>
         <v>5.8486047407303667E-4</v>
       </c>
-      <c r="D37" s="50"/>
-      <c r="E37" s="50">
+      <c r="D37" s="57"/>
+      <c r="E37" s="57">
         <f>E36+F36</f>
         <v>0.55141413267077066</v>
       </c>
-      <c r="F37" s="50"/>
-      <c r="G37" s="50">
+      <c r="F37" s="57"/>
+      <c r="G37" s="57">
         <f>G36+H36</f>
         <v>1.1049913378383109</v>
       </c>
-      <c r="H37" s="50"/>
-      <c r="I37" s="50">
+      <c r="H37" s="57"/>
+      <c r="I37" s="57">
         <f>I36+J36</f>
         <v>4.376597458072197E-2</v>
       </c>
-      <c r="J37" s="50"/>
-      <c r="K37" s="50">
+      <c r="J37" s="57"/>
+      <c r="K37" s="57">
         <f>K36+L36</f>
         <v>63.671869264221172</v>
       </c>
-      <c r="L37" s="50"/>
-      <c r="M37" s="50">
+      <c r="L37" s="57"/>
+      <c r="M37" s="57">
         <f>M36+N36</f>
         <v>5.3985522503124574</v>
       </c>
-      <c r="N37" s="50"/>
+      <c r="N37" s="57"/>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B38" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C38" s="51">
+      <c r="C38" s="58">
         <f>C26</f>
         <v>9053.1</v>
       </c>
-      <c r="D38" s="51"/>
-      <c r="E38" s="51">
+      <c r="D38" s="58"/>
+      <c r="E38" s="58">
         <f>D26</f>
         <v>829.1</v>
       </c>
-      <c r="F38" s="51"/>
-      <c r="G38" s="51">
+      <c r="F38" s="58"/>
+      <c r="G38" s="58">
         <f>E26</f>
         <v>613</v>
       </c>
-      <c r="H38" s="51"/>
-      <c r="I38" s="51">
+      <c r="H38" s="58"/>
+      <c r="I38" s="58">
         <f>F26</f>
         <v>1435</v>
       </c>
-      <c r="J38" s="51"/>
-      <c r="K38" s="51">
+      <c r="J38" s="58"/>
+      <c r="K38" s="58">
         <f>G26</f>
         <v>454.9</v>
       </c>
-      <c r="L38" s="51"/>
-      <c r="M38" s="51">
+      <c r="L38" s="58"/>
+      <c r="M38" s="58">
         <f>H26</f>
         <v>446.1</v>
       </c>
-      <c r="N38" s="51"/>
+      <c r="N38" s="58"/>
     </row>
     <row r="39" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B39" s="45" t="s">
+      <c r="B39" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="52">
+      <c r="C39" s="53">
         <f>(C37*C38+E37*E38+G37*G38+I37*I38+K37*K38+M37*M38)/SUM(C38:M38)</f>
         <v>2.5387542559177616</v>
       </c>
-      <c r="D39" s="53"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="53"/>
-      <c r="G39" s="53"/>
-      <c r="H39" s="53"/>
-      <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="53"/>
-      <c r="L39" s="53"/>
-      <c r="M39" s="53"/>
-      <c r="N39" s="54"/>
+      <c r="D39" s="54"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="54"/>
+      <c r="I39" s="54"/>
+      <c r="J39" s="54"/>
+      <c r="K39" s="54"/>
+      <c r="L39" s="54"/>
+      <c r="M39" s="54"/>
+      <c r="N39" s="55"/>
     </row>
     <row r="42" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B42" s="42" t="s">
+      <c r="B42" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="C42" s="42"/>
-      <c r="D42" s="42"/>
-      <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
-      <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
-      <c r="M42" s="42"/>
-      <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
-      <c r="Q42" s="42"/>
+      <c r="C42" s="56"/>
+      <c r="D42" s="56"/>
+      <c r="E42" s="56"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="56"/>
+      <c r="H42" s="56"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="56"/>
+      <c r="K42" s="56"/>
+      <c r="L42" s="56"/>
+      <c r="M42" s="56"/>
+      <c r="N42" s="56"/>
+      <c r="O42" s="56"/>
+      <c r="P42" s="56"/>
+      <c r="Q42" s="56"/>
     </row>
     <row r="44" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B44" s="39" t="s">
+      <c r="B44" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="C44" s="39"/>
-      <c r="D44" s="55">
+      <c r="C44" s="46"/>
+      <c r="D44" s="33">
         <f>C39</f>
         <v>2.5387542559177616</v>
       </c>
-      <c r="I44" s="71" t="s">
+      <c r="I44" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="J44" s="71"/>
-      <c r="K44" s="39"/>
-      <c r="L44" s="40">
+      <c r="J44" s="45"/>
+      <c r="K44" s="46"/>
+      <c r="L44" s="27">
         <f>SUM(D26:H26)</f>
         <v>3778.1</v>
       </c>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B45" s="39" t="s">
+      <c r="B45" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="C45" s="39"/>
+      <c r="C45" s="46"/>
       <c r="D45" s="1">
         <v>0.6</v>
       </c>
       <c r="E45" t="s">
         <v>61</v>
       </c>
-      <c r="I45" s="71" t="s">
+      <c r="I45" s="45" t="s">
         <v>66</v>
       </c>
-      <c r="J45" s="71"/>
-      <c r="K45" s="39"/>
+      <c r="J45" s="45"/>
+      <c r="K45" s="46"/>
       <c r="L45">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B46" s="59" t="s">
+      <c r="B46" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C46" s="59"/>
+      <c r="C46" s="47"/>
       <c r="D46">
         <v>20</v>
       </c>
-      <c r="I46" s="43" t="s">
+      <c r="I46" t="s">
         <v>95</v>
       </c>
-      <c r="J46" s="43"/>
       <c r="K46" s="3"/>
     </row>
     <row r="47" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B47" s="59" t="s">
+      <c r="B47" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="C47" s="59"/>
-      <c r="D47" s="56">
+      <c r="C47" s="47"/>
+      <c r="D47" s="34">
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="E47" t="s">
@@ -2715,79 +2741,78 @@
         <v>96</v>
       </c>
       <c r="K47" s="3"/>
-      <c r="L47" s="72">
+      <c r="L47" s="40">
         <v>0.03</v>
       </c>
-      <c r="O47" s="3"/>
     </row>
     <row r="48" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B48" s="39" t="s">
+      <c r="B48" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="39"/>
-      <c r="D48" s="47">
+      <c r="C48" s="46"/>
+      <c r="D48" s="31">
         <v>9</v>
       </c>
-      <c r="I48" s="71" t="s">
+      <c r="I48" s="45" t="s">
         <v>97</v>
       </c>
-      <c r="J48" s="71"/>
-      <c r="K48" s="39"/>
-      <c r="L48" s="56">
+      <c r="J48" s="45"/>
+      <c r="K48" s="46"/>
+      <c r="L48" s="34">
         <v>0.115</v>
       </c>
     </row>
     <row r="50" spans="2:17" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B50" s="42" t="s">
+      <c r="B50" s="56" t="s">
         <v>73</v>
       </c>
-      <c r="C50" s="42"/>
-      <c r="D50" s="42"/>
-      <c r="E50" s="42"/>
-      <c r="F50" s="42"/>
-      <c r="G50" s="42"/>
-      <c r="H50" s="42"/>
-      <c r="I50" s="42"/>
-      <c r="J50" s="42"/>
-      <c r="K50" s="42"/>
-      <c r="L50" s="42"/>
-      <c r="M50" s="42"/>
-      <c r="N50" s="42"/>
-      <c r="O50" s="42"/>
-      <c r="P50" s="42"/>
-      <c r="Q50" s="42"/>
+      <c r="C50" s="56"/>
+      <c r="D50" s="56"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="56"/>
+      <c r="G50" s="56"/>
+      <c r="H50" s="56"/>
+      <c r="I50" s="56"/>
+      <c r="J50" s="56"/>
+      <c r="K50" s="56"/>
+      <c r="L50" s="56"/>
+      <c r="M50" s="56"/>
+      <c r="N50" s="56"/>
+      <c r="O50" s="56"/>
+      <c r="P50" s="56"/>
+      <c r="Q50" s="56"/>
     </row>
     <row r="51" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B51" s="57" t="s">
+      <c r="B51" s="44" t="s">
         <v>69</v>
       </c>
-      <c r="C51" s="57"/>
-      <c r="D51" s="57"/>
-      <c r="E51" s="57"/>
-      <c r="F51" s="57"/>
-      <c r="G51" s="57"/>
-      <c r="H51" s="57"/>
-      <c r="I51" s="57"/>
-      <c r="J51" s="57"/>
-      <c r="K51" s="57"/>
-      <c r="L51" s="57"/>
-      <c r="M51" s="57"/>
-      <c r="N51" s="57"/>
-      <c r="O51" s="57"/>
-      <c r="P51" s="57"/>
-      <c r="Q51" s="57"/>
+      <c r="C51" s="44"/>
+      <c r="D51" s="44"/>
+      <c r="E51" s="44"/>
+      <c r="F51" s="44"/>
+      <c r="G51" s="44"/>
+      <c r="H51" s="44"/>
+      <c r="I51" s="44"/>
+      <c r="J51" s="44"/>
+      <c r="K51" s="44"/>
+      <c r="L51" s="44"/>
+      <c r="M51" s="44"/>
+      <c r="N51" s="44"/>
+      <c r="O51" s="44"/>
+      <c r="P51" s="44"/>
+      <c r="Q51" s="44"/>
     </row>
     <row r="52" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>70</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="27">
         <f>L44*(1+D47)^L45</f>
         <v>4366.0668124999993</v>
       </c>
     </row>
     <row r="53" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B53" s="58" t="s">
+      <c r="B53" s="35" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2795,30 +2820,30 @@
       <c r="B54" t="s">
         <v>72</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="33">
         <f>365*C52*((1+D47)^D46-1)*D44*D45/D47/1000000</f>
         <v>105.12112589208186</v>
       </c>
     </row>
     <row r="56" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B56" s="57" t="s">
+      <c r="B56" s="44" t="s">
         <v>74</v>
       </c>
-      <c r="C56" s="57"/>
-      <c r="D56" s="57"/>
-      <c r="E56" s="57"/>
-      <c r="F56" s="57"/>
-      <c r="G56" s="57"/>
-      <c r="H56" s="57"/>
-      <c r="I56" s="57"/>
-      <c r="J56" s="57"/>
-      <c r="K56" s="57"/>
-      <c r="L56" s="57"/>
-      <c r="M56" s="57"/>
-      <c r="N56" s="57"/>
-      <c r="O56" s="57"/>
-      <c r="P56" s="57"/>
-      <c r="Q56" s="57"/>
+      <c r="C56" s="44"/>
+      <c r="D56" s="44"/>
+      <c r="E56" s="44"/>
+      <c r="F56" s="44"/>
+      <c r="G56" s="44"/>
+      <c r="H56" s="44"/>
+      <c r="I56" s="44"/>
+      <c r="J56" s="44"/>
+      <c r="K56" s="44"/>
+      <c r="L56" s="44"/>
+      <c r="M56" s="44"/>
+      <c r="N56" s="44"/>
+      <c r="O56" s="44"/>
+      <c r="P56" s="44"/>
+      <c r="Q56" s="44"/>
     </row>
     <row r="57" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B57" s="5" t="s">
@@ -2874,127 +2899,127 @@
       </c>
     </row>
     <row r="65" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B65" s="57" t="s">
+      <c r="B65" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="C65" s="57"/>
-      <c r="D65" s="57"/>
-      <c r="E65" s="57"/>
-      <c r="F65" s="57"/>
-      <c r="G65" s="57"/>
-      <c r="H65" s="57"/>
-      <c r="I65" s="57"/>
-      <c r="J65" s="57"/>
-      <c r="K65" s="57"/>
-      <c r="L65" s="57"/>
-      <c r="M65" s="57"/>
-      <c r="N65" s="57"/>
-      <c r="O65" s="57"/>
-      <c r="P65" s="57"/>
-      <c r="Q65" s="57"/>
+      <c r="C65" s="44"/>
+      <c r="D65" s="44"/>
+      <c r="E65" s="44"/>
+      <c r="F65" s="44"/>
+      <c r="G65" s="44"/>
+      <c r="H65" s="44"/>
+      <c r="I65" s="44"/>
+      <c r="J65" s="44"/>
+      <c r="K65" s="44"/>
+      <c r="L65" s="44"/>
+      <c r="M65" s="44"/>
+      <c r="N65" s="44"/>
+      <c r="O65" s="44"/>
+      <c r="P65" s="44"/>
+      <c r="Q65" s="44"/>
     </row>
     <row r="69" spans="2:17" ht="18" x14ac:dyDescent="0.35">
-      <c r="E69" s="61" t="s">
+      <c r="E69" s="48" t="s">
         <v>75</v>
       </c>
-      <c r="F69" s="61"/>
-      <c r="G69" s="61" t="s">
+      <c r="F69" s="48"/>
+      <c r="G69" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="H69" s="61"/>
+      <c r="H69" s="48"/>
     </row>
     <row r="70" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E70" s="62" t="s">
+      <c r="E70" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="F70" s="62"/>
-      <c r="G70" s="63">
+      <c r="F70" s="49"/>
+      <c r="G70" s="52">
         <f>C58+C59</f>
         <v>160</v>
       </c>
-      <c r="H70" s="63"/>
+      <c r="H70" s="52"/>
     </row>
     <row r="71" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E71" s="62"/>
-      <c r="F71" s="62"/>
-      <c r="G71" s="63"/>
-      <c r="H71" s="63"/>
+      <c r="E71" s="49"/>
+      <c r="F71" s="49"/>
+      <c r="G71" s="52"/>
+      <c r="H71" s="52"/>
     </row>
     <row r="72" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E72" s="64" t="s">
+      <c r="E72" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="F72" s="64"/>
-      <c r="G72" s="63">
+      <c r="F72" s="50"/>
+      <c r="G72" s="52">
         <f>C60+C61</f>
         <v>450</v>
       </c>
-      <c r="H72" s="63"/>
+      <c r="H72" s="52"/>
     </row>
     <row r="73" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E73" s="64"/>
-      <c r="F73" s="64"/>
-      <c r="G73" s="63"/>
-      <c r="H73" s="63"/>
+      <c r="E73" s="50"/>
+      <c r="F73" s="50"/>
+      <c r="G73" s="52"/>
+      <c r="H73" s="52"/>
     </row>
     <row r="74" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E74" s="64"/>
-      <c r="F74" s="64"/>
-      <c r="G74" s="63"/>
-      <c r="H74" s="63"/>
+      <c r="E74" s="50"/>
+      <c r="F74" s="50"/>
+      <c r="G74" s="52"/>
+      <c r="H74" s="52"/>
     </row>
     <row r="75" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E75" s="65" t="s">
+      <c r="E75" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="F75" s="65"/>
-      <c r="G75" s="63">
+      <c r="F75" s="51"/>
+      <c r="G75" s="52">
         <f>C62</f>
         <v>500</v>
       </c>
-      <c r="H75" s="63"/>
+      <c r="H75" s="52"/>
     </row>
     <row r="76" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E76" s="65"/>
-      <c r="F76" s="65"/>
-      <c r="G76" s="63"/>
-      <c r="H76" s="63"/>
+      <c r="E76" s="51"/>
+      <c r="F76" s="51"/>
+      <c r="G76" s="52"/>
+      <c r="H76" s="52"/>
     </row>
     <row r="77" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E77" s="65"/>
-      <c r="F77" s="65"/>
-      <c r="G77" s="63"/>
-      <c r="H77" s="63"/>
+      <c r="E77" s="51"/>
+      <c r="F77" s="51"/>
+      <c r="G77" s="52"/>
+      <c r="H77" s="52"/>
     </row>
     <row r="78" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="E78" s="65"/>
-      <c r="F78" s="65"/>
-      <c r="G78" s="63"/>
-      <c r="H78" s="63"/>
+      <c r="E78" s="51"/>
+      <c r="F78" s="51"/>
+      <c r="G78" s="52"/>
+      <c r="H78" s="52"/>
     </row>
     <row r="80" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B80" s="57" t="s">
+      <c r="B80" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="C80" s="57"/>
-      <c r="D80" s="57"/>
-      <c r="E80" s="57"/>
-      <c r="F80" s="57"/>
-      <c r="G80" s="57"/>
-      <c r="H80" s="57"/>
-      <c r="I80" s="57"/>
-      <c r="J80" s="57"/>
-      <c r="K80" s="57"/>
-      <c r="L80" s="57"/>
-      <c r="M80" s="57"/>
-      <c r="N80" s="57"/>
-      <c r="O80" s="57"/>
-      <c r="P80" s="57"/>
-      <c r="Q80" s="57"/>
+      <c r="C80" s="44"/>
+      <c r="D80" s="44"/>
+      <c r="E80" s="44"/>
+      <c r="F80" s="44"/>
+      <c r="G80" s="44"/>
+      <c r="H80" s="44"/>
+      <c r="I80" s="44"/>
+      <c r="J80" s="44"/>
+      <c r="K80" s="44"/>
+      <c r="L80" s="44"/>
+      <c r="M80" s="44"/>
+      <c r="N80" s="44"/>
+      <c r="O80" s="44"/>
+      <c r="P80" s="44"/>
+      <c r="Q80" s="44"/>
     </row>
     <row r="81" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B81" s="24"/>
-      <c r="C81" s="60" t="s">
+      <c r="C81" s="36" t="s">
         <v>64</v>
       </c>
       <c r="D81" s="26" t="s">
@@ -3005,7 +3030,7 @@
       <c r="B82" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="C82" s="69" cm="1">
+      <c r="C82" s="38" cm="1">
         <f t="array" ref="C82">17.6*(cbr)^0.64</f>
         <v>71.817101600169877</v>
       </c>
@@ -3017,7 +3042,7 @@
       <c r="B83" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C83" s="48">
+      <c r="C83" s="32">
         <f>0.2*($G$72)^0.45*C82</f>
         <v>224.49336032364351</v>
       </c>
@@ -3029,7 +3054,7 @@
       <c r="B84" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="C84" s="70">
+      <c r="C84" s="39">
         <v>2200</v>
       </c>
       <c r="D84" s="23">
@@ -3037,27 +3062,27 @@
       </c>
     </row>
     <row r="86" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B86" s="57" t="s">
+      <c r="B86" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="C86" s="57"/>
-      <c r="D86" s="57"/>
-      <c r="E86" s="57"/>
-      <c r="F86" s="57"/>
-      <c r="G86" s="57"/>
-      <c r="H86" s="57"/>
-      <c r="I86" s="57"/>
-      <c r="J86" s="57"/>
-      <c r="K86" s="57"/>
-      <c r="L86" s="57"/>
-      <c r="M86" s="57"/>
-      <c r="N86" s="57"/>
-      <c r="O86" s="57"/>
-      <c r="P86" s="57"/>
-      <c r="Q86" s="57"/>
+      <c r="C86" s="44"/>
+      <c r="D86" s="44"/>
+      <c r="E86" s="44"/>
+      <c r="F86" s="44"/>
+      <c r="G86" s="44"/>
+      <c r="H86" s="44"/>
+      <c r="I86" s="44"/>
+      <c r="J86" s="44"/>
+      <c r="K86" s="44"/>
+      <c r="L86" s="44"/>
+      <c r="M86" s="44"/>
+      <c r="N86" s="44"/>
+      <c r="O86" s="44"/>
+      <c r="P86" s="44"/>
+      <c r="Q86" s="44"/>
     </row>
     <row r="87" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B87" s="58" t="s">
+      <c r="B87" s="35" t="s">
         <v>88</v>
       </c>
       <c r="N87" t="s">
@@ -3065,10 +3090,10 @@
       </c>
     </row>
     <row r="88" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B88" s="66" t="s">
+      <c r="B88" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="C88" s="67">
+      <c r="C88" s="43">
         <f>(1.41*(10^(-8))/($C$54*1000000))^(1/4.5337)</f>
         <v>3.1550251481005814E-4</v>
       </c>
@@ -3077,22 +3102,22 @@
       </c>
     </row>
     <row r="90" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B90" s="58" t="s">
+      <c r="B90" s="35" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="91" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B91" s="66" t="s">
+      <c r="B91" s="42" t="s">
         <v>92</v>
       </c>
-      <c r="C91" s="67">
+      <c r="C91" s="43">
         <f>(0.5161*F92*0.0001/($C$54*1000000*($C$84^0.854)))^(1/3.89)</f>
         <v>1.6991843829641307E-4</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="F91" s="68">
+      <c r="F91" s="37">
         <f>4.84*(L48/(L48+L47)-0.69)</f>
         <v>0.49902068965517227</v>
       </c>
@@ -3101,55 +3126,53 @@
       <c r="E92" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F92" s="68">
+      <c r="F92" s="37">
         <f>10^F91</f>
         <v>3.1551549304020763</v>
       </c>
     </row>
     <row r="95" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B95" s="57" t="s">
+      <c r="B95" s="44" t="s">
         <v>93</v>
       </c>
-      <c r="C95" s="57"/>
-      <c r="D95" s="57"/>
-      <c r="E95" s="57"/>
-      <c r="F95" s="57"/>
-      <c r="G95" s="57"/>
-      <c r="H95" s="57"/>
-      <c r="I95" s="57"/>
-      <c r="J95" s="57"/>
-      <c r="K95" s="57"/>
-      <c r="L95" s="57"/>
-      <c r="M95" s="57"/>
-      <c r="N95" s="57"/>
-      <c r="O95" s="57"/>
-      <c r="P95" s="57"/>
-      <c r="Q95" s="57"/>
+      <c r="C95" s="44"/>
+      <c r="D95" s="44"/>
+      <c r="E95" s="44"/>
+      <c r="F95" s="44"/>
+      <c r="G95" s="44"/>
+      <c r="H95" s="44"/>
+      <c r="I95" s="44"/>
+      <c r="J95" s="44"/>
+      <c r="K95" s="44"/>
+      <c r="L95" s="44"/>
+      <c r="M95" s="44"/>
+      <c r="N95" s="44"/>
+      <c r="O95" s="44"/>
+      <c r="P95" s="44"/>
+      <c r="Q95" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="57">
-    <mergeCell ref="B80:Q80"/>
-    <mergeCell ref="B86:Q86"/>
-    <mergeCell ref="B95:Q95"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="I45:K45"/>
-    <mergeCell ref="C39:N39"/>
-    <mergeCell ref="B42:Q42"/>
-    <mergeCell ref="B51:Q51"/>
-    <mergeCell ref="B50:Q50"/>
-    <mergeCell ref="B56:Q56"/>
-    <mergeCell ref="B65:Q65"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="E70:F71"/>
-    <mergeCell ref="E72:F74"/>
-    <mergeCell ref="E75:F78"/>
-    <mergeCell ref="G70:H71"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="M32:N32"/>
+    <mergeCell ref="B30:Q30"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="I33:J33"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="M33:N33"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="I32:J32"/>
     <mergeCell ref="G72:H74"/>
     <mergeCell ref="G75:H78"/>
     <mergeCell ref="B44:C44"/>
@@ -3165,26 +3188,28 @@
     <mergeCell ref="G37:H37"/>
     <mergeCell ref="I37:J37"/>
     <mergeCell ref="K37:L37"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="M32:N32"/>
-    <mergeCell ref="B30:Q30"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="M33:N33"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="I45:K45"/>
+    <mergeCell ref="C39:N39"/>
+    <mergeCell ref="B42:Q42"/>
+    <mergeCell ref="B51:Q51"/>
+    <mergeCell ref="B50:Q50"/>
+    <mergeCell ref="B80:Q80"/>
+    <mergeCell ref="B86:Q86"/>
+    <mergeCell ref="B95:Q95"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B56:Q56"/>
+    <mergeCell ref="B65:Q65"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="E70:F71"/>
+    <mergeCell ref="E72:F74"/>
+    <mergeCell ref="E75:F78"/>
+    <mergeCell ref="G70:H71"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3213,64 +3238,64 @@
   </cols>
   <sheetData>
     <row r="6" spans="2:26" ht="18" x14ac:dyDescent="0.3">
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="66" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
-      <c r="O6" s="31" t="s">
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="66"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66"/>
+      <c r="K6" s="66"/>
+      <c r="L6" s="66"/>
+      <c r="M6" s="66"/>
+      <c r="O6" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
-      <c r="R6" s="31"/>
-      <c r="S6" s="31"/>
-      <c r="T6" s="31"/>
-      <c r="U6" s="31"/>
-      <c r="V6" s="31"/>
-      <c r="W6" s="31"/>
-      <c r="X6" s="31"/>
-      <c r="Y6" s="31"/>
-      <c r="Z6" s="31"/>
+      <c r="P6" s="66"/>
+      <c r="Q6" s="66"/>
+      <c r="R6" s="66"/>
+      <c r="S6" s="66"/>
+      <c r="T6" s="66"/>
+      <c r="U6" s="66"/>
+      <c r="V6" s="66"/>
+      <c r="W6" s="66"/>
+      <c r="X6" s="66"/>
+      <c r="Y6" s="66"/>
+      <c r="Z6" s="66"/>
     </row>
     <row r="8" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
-      <c r="O8" s="32" t="s">
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="64"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="64"/>
+      <c r="M8" s="64"/>
+      <c r="O8" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="P8" s="32"/>
-      <c r="Q8" s="32"/>
-      <c r="R8" s="32"/>
-      <c r="S8" s="32"/>
-      <c r="T8" s="32"/>
-      <c r="U8" s="32"/>
-      <c r="V8" s="32"/>
-      <c r="W8" s="32"/>
-      <c r="X8" s="32"/>
-      <c r="Y8" s="32"/>
-      <c r="Z8" s="32"/>
+      <c r="P8" s="64"/>
+      <c r="Q8" s="64"/>
+      <c r="R8" s="64"/>
+      <c r="S8" s="64"/>
+      <c r="T8" s="64"/>
+      <c r="U8" s="64"/>
+      <c r="V8" s="64"/>
+      <c r="W8" s="64"/>
+      <c r="X8" s="64"/>
+      <c r="Y8" s="64"/>
+      <c r="Z8" s="64"/>
     </row>
     <row r="9" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B9" s="24" t="s">
@@ -3280,17 +3305,17 @@
         <v>94.5</v>
       </c>
       <c r="D9" s="25"/>
-      <c r="E9" s="33" t="s">
+      <c r="E9" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="34"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="67"/>
+      <c r="H9" s="67"/>
+      <c r="I9" s="67"/>
+      <c r="J9" s="67"/>
+      <c r="K9" s="67"/>
+      <c r="L9" s="67"/>
+      <c r="M9" s="68"/>
       <c r="O9" s="24" t="s">
         <v>26</v>
       </c>
@@ -3298,36 +3323,35 @@
         <v>94.5</v>
       </c>
       <c r="Q9" s="25"/>
-      <c r="R9" s="33" t="s">
+      <c r="R9" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="S9" s="33"/>
-      <c r="T9" s="33"/>
-      <c r="U9" s="33"/>
-      <c r="V9" s="33"/>
-      <c r="W9" s="33"/>
-      <c r="X9" s="33"/>
-      <c r="Y9" s="33"/>
-      <c r="Z9" s="34"/>
+      <c r="S9" s="67"/>
+      <c r="T9" s="67"/>
+      <c r="U9" s="67"/>
+      <c r="V9" s="67"/>
+      <c r="W9" s="67"/>
+      <c r="X9" s="67"/>
+      <c r="Y9" s="67"/>
+      <c r="Z9" s="68"/>
     </row>
     <row r="10" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="43">
+      <c r="C10">
         <f>3.5*6+2*(1.5+2)+2.5+0.5*2</f>
         <v>31.5</v>
       </c>
-      <c r="D10" s="43"/>
-      <c r="E10" s="73"/>
-      <c r="F10" s="73"/>
-      <c r="G10" s="73"/>
-      <c r="H10" s="73"/>
-      <c r="I10" s="73"/>
-      <c r="J10" s="73"/>
-      <c r="K10" s="73"/>
-      <c r="L10" s="73"/>
-      <c r="M10" s="36"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="69"/>
+      <c r="K10" s="69"/>
+      <c r="L10" s="69"/>
+      <c r="M10" s="70"/>
       <c r="O10" s="4" t="s">
         <v>27</v>
       </c>
@@ -3335,112 +3359,89 @@
         <f>3.5*6+2*(1.5+2)+2.5+0.5*2</f>
         <v>31.5</v>
       </c>
-      <c r="R10" s="35"/>
-      <c r="S10" s="35"/>
-      <c r="T10" s="35"/>
-      <c r="U10" s="35"/>
-      <c r="V10" s="35"/>
-      <c r="W10" s="35"/>
-      <c r="X10" s="35"/>
-      <c r="Y10" s="35"/>
-      <c r="Z10" s="36"/>
+      <c r="R10" s="69"/>
+      <c r="S10" s="69"/>
+      <c r="T10" s="69"/>
+      <c r="U10" s="69"/>
+      <c r="V10" s="69"/>
+      <c r="W10" s="69"/>
+      <c r="X10" s="69"/>
+      <c r="Y10" s="69"/>
+      <c r="Z10" s="70"/>
     </row>
     <row r="11" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B11" s="4"/>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="73"/>
-      <c r="J11" s="73"/>
-      <c r="K11" s="73"/>
-      <c r="L11" s="73"/>
-      <c r="M11" s="36"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="69"/>
+      <c r="L11" s="69"/>
+      <c r="M11" s="70"/>
       <c r="O11" s="4"/>
-      <c r="R11" s="35"/>
-      <c r="S11" s="35"/>
-      <c r="T11" s="35"/>
-      <c r="U11" s="35"/>
-      <c r="V11" s="35"/>
-      <c r="W11" s="35"/>
-      <c r="X11" s="35"/>
-      <c r="Y11" s="35"/>
-      <c r="Z11" s="36"/>
+      <c r="R11" s="69"/>
+      <c r="S11" s="69"/>
+      <c r="T11" s="69"/>
+      <c r="U11" s="69"/>
+      <c r="V11" s="69"/>
+      <c r="W11" s="69"/>
+      <c r="X11" s="69"/>
+      <c r="Y11" s="69"/>
+      <c r="Z11" s="70"/>
     </row>
     <row r="12" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B12" s="4"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="73"/>
-      <c r="F12" s="73"/>
-      <c r="G12" s="73"/>
-      <c r="H12" s="73"/>
-      <c r="I12" s="73"/>
-      <c r="J12" s="73"/>
-      <c r="K12" s="73"/>
-      <c r="L12" s="73"/>
-      <c r="M12" s="36"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="69"/>
+      <c r="H12" s="69"/>
+      <c r="I12" s="69"/>
+      <c r="J12" s="69"/>
+      <c r="K12" s="69"/>
+      <c r="L12" s="69"/>
+      <c r="M12" s="70"/>
       <c r="O12" s="4"/>
-      <c r="R12" s="35"/>
-      <c r="S12" s="35"/>
-      <c r="T12" s="35"/>
-      <c r="U12" s="35"/>
-      <c r="V12" s="35"/>
-      <c r="W12" s="35"/>
-      <c r="X12" s="35"/>
-      <c r="Y12" s="35"/>
-      <c r="Z12" s="36"/>
+      <c r="R12" s="69"/>
+      <c r="S12" s="69"/>
+      <c r="T12" s="69"/>
+      <c r="U12" s="69"/>
+      <c r="V12" s="69"/>
+      <c r="W12" s="69"/>
+      <c r="X12" s="69"/>
+      <c r="Y12" s="69"/>
+      <c r="Z12" s="70"/>
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
       <c r="M13" s="3"/>
-      <c r="O13" s="37" t="s">
+      <c r="O13" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="P13" s="38"/>
-      <c r="Q13" s="38"/>
-      <c r="R13" s="38"/>
-      <c r="S13" s="38"/>
-      <c r="T13" s="38"/>
-      <c r="U13" s="38"/>
-      <c r="V13" s="38"/>
-      <c r="W13" s="38"/>
-      <c r="X13" s="38"/>
-      <c r="Y13" s="38"/>
-      <c r="Z13" s="39"/>
+      <c r="P13" s="45"/>
+      <c r="Q13" s="45"/>
+      <c r="R13" s="45"/>
+      <c r="S13" s="45"/>
+      <c r="T13" s="45"/>
+      <c r="U13" s="45"/>
+      <c r="V13" s="45"/>
+      <c r="W13" s="45"/>
+      <c r="X13" s="45"/>
+      <c r="Y13" s="45"/>
+      <c r="Z13" s="46"/>
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="str">
         <f>'Flexible Pavement Design'!B57</f>
         <v>Layer</v>
       </c>
-      <c r="C14" s="43" t="str">
+      <c r="C14" t="str">
         <f>'Flexible Pavement Design'!C57</f>
         <v>Thickness (in mm)</v>
       </c>
-      <c r="D14" s="43"/>
-      <c r="E14" s="43"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="43"/>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
       <c r="M14" s="3"/>
       <c r="O14" s="4" t="s">
         <v>33</v>
@@ -3455,19 +3456,10 @@
         <f>'Flexible Pavement Design'!B58</f>
         <v>BC (Surface Layer)</v>
       </c>
-      <c r="C15" s="43">
+      <c r="C15">
         <f>'Flexible Pavement Design'!C58</f>
         <v>40</v>
       </c>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="43"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="43"/>
       <c r="M15" s="3"/>
       <c r="O15" s="4" t="s">
         <v>34</v>
@@ -3482,19 +3474,10 @@
         <f>'Flexible Pavement Design'!B59</f>
         <v>Binder coarse</v>
       </c>
-      <c r="C16" s="43">
+      <c r="C16">
         <f>'Flexible Pavement Design'!C59</f>
         <v>120</v>
       </c>
-      <c r="D16" s="43"/>
-      <c r="E16" s="43"/>
-      <c r="F16" s="43"/>
-      <c r="G16" s="43"/>
-      <c r="H16" s="43"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="43"/>
-      <c r="L16" s="43"/>
       <c r="M16" s="3"/>
       <c r="O16" s="4" t="s">
         <v>35</v>
@@ -3509,19 +3492,10 @@
         <f>'Flexible Pavement Design'!B60</f>
         <v>Base (WMM)</v>
       </c>
-      <c r="C17" s="43">
+      <c r="C17">
         <f>'Flexible Pavement Design'!C60</f>
         <v>250</v>
       </c>
-      <c r="D17" s="43"/>
-      <c r="E17" s="43"/>
-      <c r="F17" s="43"/>
-      <c r="G17" s="43"/>
-      <c r="H17" s="43"/>
-      <c r="I17" s="43"/>
-      <c r="J17" s="43"/>
-      <c r="K17" s="43"/>
-      <c r="L17" s="43"/>
       <c r="M17" s="3"/>
       <c r="O17" s="4" t="s">
         <v>36</v>
@@ -3568,34 +3542,34 @@
       <c r="Z18" s="23"/>
     </row>
     <row r="21" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
-      <c r="L21" s="32"/>
-      <c r="M21" s="32"/>
-      <c r="O21" s="32" t="s">
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
+      <c r="E21" s="64"/>
+      <c r="F21" s="64"/>
+      <c r="G21" s="64"/>
+      <c r="H21" s="64"/>
+      <c r="I21" s="64"/>
+      <c r="J21" s="64"/>
+      <c r="K21" s="64"/>
+      <c r="L21" s="64"/>
+      <c r="M21" s="64"/>
+      <c r="O21" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="P21" s="32"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="32"/>
-      <c r="T21" s="32"/>
-      <c r="U21" s="32"/>
-      <c r="V21" s="32"/>
-      <c r="W21" s="32"/>
-      <c r="X21" s="32"/>
-      <c r="Y21" s="32"/>
-      <c r="Z21" s="32"/>
+      <c r="P21" s="64"/>
+      <c r="Q21" s="64"/>
+      <c r="R21" s="64"/>
+      <c r="S21" s="64"/>
+      <c r="T21" s="64"/>
+      <c r="U21" s="64"/>
+      <c r="V21" s="64"/>
+      <c r="W21" s="64"/>
+      <c r="X21" s="64"/>
+      <c r="Y21" s="64"/>
+      <c r="Z21" s="64"/>
     </row>
     <row r="22" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B22" s="24"/>
@@ -3692,34 +3666,34 @@
       <c r="Z30" s="23"/>
     </row>
     <row r="33" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
-      <c r="E33" s="32"/>
-      <c r="F33" s="32"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="32"/>
-      <c r="J33" s="32"/>
-      <c r="K33" s="32"/>
-      <c r="L33" s="32"/>
-      <c r="M33" s="32"/>
-      <c r="O33" s="32" t="s">
+      <c r="C33" s="64"/>
+      <c r="D33" s="64"/>
+      <c r="E33" s="64"/>
+      <c r="F33" s="64"/>
+      <c r="G33" s="64"/>
+      <c r="H33" s="64"/>
+      <c r="I33" s="64"/>
+      <c r="J33" s="64"/>
+      <c r="K33" s="64"/>
+      <c r="L33" s="64"/>
+      <c r="M33" s="64"/>
+      <c r="O33" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="P33" s="32"/>
-      <c r="Q33" s="32"/>
-      <c r="R33" s="32"/>
-      <c r="S33" s="32"/>
-      <c r="T33" s="32"/>
-      <c r="U33" s="32"/>
-      <c r="V33" s="32"/>
-      <c r="W33" s="32"/>
-      <c r="X33" s="32"/>
-      <c r="Y33" s="32"/>
-      <c r="Z33" s="32"/>
+      <c r="P33" s="64"/>
+      <c r="Q33" s="64"/>
+      <c r="R33" s="64"/>
+      <c r="S33" s="64"/>
+      <c r="T33" s="64"/>
+      <c r="U33" s="64"/>
+      <c r="V33" s="64"/>
+      <c r="W33" s="64"/>
+      <c r="X33" s="64"/>
+      <c r="Y33" s="64"/>
+      <c r="Z33" s="64"/>
     </row>
     <row r="34" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B34" s="24"/>
@@ -3840,34 +3814,34 @@
       <c r="Z46" s="23"/>
     </row>
     <row r="49" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B49" s="32" t="s">
+      <c r="B49" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="C49" s="32"/>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="32"/>
-      <c r="I49" s="32"/>
-      <c r="J49" s="32"/>
-      <c r="K49" s="32"/>
-      <c r="L49" s="32"/>
-      <c r="M49" s="32"/>
-      <c r="O49" s="32" t="s">
+      <c r="C49" s="64"/>
+      <c r="D49" s="64"/>
+      <c r="E49" s="64"/>
+      <c r="F49" s="64"/>
+      <c r="G49" s="64"/>
+      <c r="H49" s="64"/>
+      <c r="I49" s="64"/>
+      <c r="J49" s="64"/>
+      <c r="K49" s="64"/>
+      <c r="L49" s="64"/>
+      <c r="M49" s="64"/>
+      <c r="O49" s="64" t="s">
         <v>40</v>
       </c>
-      <c r="P49" s="32"/>
-      <c r="Q49" s="32"/>
-      <c r="R49" s="32"/>
-      <c r="S49" s="32"/>
-      <c r="T49" s="32"/>
-      <c r="U49" s="32"/>
-      <c r="V49" s="32"/>
-      <c r="W49" s="32"/>
-      <c r="X49" s="32"/>
-      <c r="Y49" s="32"/>
-      <c r="Z49" s="32"/>
+      <c r="P49" s="64"/>
+      <c r="Q49" s="64"/>
+      <c r="R49" s="64"/>
+      <c r="S49" s="64"/>
+      <c r="T49" s="64"/>
+      <c r="U49" s="64"/>
+      <c r="V49" s="64"/>
+      <c r="W49" s="64"/>
+      <c r="X49" s="64"/>
+      <c r="Y49" s="64"/>
+      <c r="Z49" s="64"/>
     </row>
     <row r="50" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B50" s="24"/>
@@ -3988,34 +3962,34 @@
       <c r="Z62" s="23"/>
     </row>
     <row r="65" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B65" s="32" t="s">
+      <c r="B65" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="C65" s="32"/>
-      <c r="D65" s="32"/>
-      <c r="E65" s="32"/>
-      <c r="F65" s="32"/>
-      <c r="G65" s="32"/>
-      <c r="H65" s="32"/>
-      <c r="I65" s="32"/>
-      <c r="J65" s="32"/>
-      <c r="K65" s="32"/>
-      <c r="L65" s="32"/>
-      <c r="M65" s="32"/>
-      <c r="O65" s="32" t="s">
+      <c r="C65" s="64"/>
+      <c r="D65" s="64"/>
+      <c r="E65" s="64"/>
+      <c r="F65" s="64"/>
+      <c r="G65" s="64"/>
+      <c r="H65" s="64"/>
+      <c r="I65" s="64"/>
+      <c r="J65" s="64"/>
+      <c r="K65" s="64"/>
+      <c r="L65" s="64"/>
+      <c r="M65" s="64"/>
+      <c r="O65" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="P65" s="32"/>
-      <c r="Q65" s="32"/>
-      <c r="R65" s="32"/>
-      <c r="S65" s="32"/>
-      <c r="T65" s="32"/>
-      <c r="U65" s="32"/>
-      <c r="V65" s="32"/>
-      <c r="W65" s="32"/>
-      <c r="X65" s="32"/>
-      <c r="Y65" s="32"/>
-      <c r="Z65" s="32"/>
+      <c r="P65" s="64"/>
+      <c r="Q65" s="64"/>
+      <c r="R65" s="64"/>
+      <c r="S65" s="64"/>
+      <c r="T65" s="64"/>
+      <c r="U65" s="64"/>
+      <c r="V65" s="64"/>
+      <c r="W65" s="64"/>
+      <c r="X65" s="64"/>
+      <c r="Y65" s="64"/>
+      <c r="Z65" s="64"/>
     </row>
     <row r="66" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B66" s="24"/>
@@ -4136,34 +4110,34 @@
       <c r="Z78" s="23"/>
     </row>
     <row r="80" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B80" s="32" t="s">
+      <c r="B80" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="C80" s="32"/>
-      <c r="D80" s="32"/>
-      <c r="E80" s="32"/>
-      <c r="F80" s="32"/>
-      <c r="G80" s="32"/>
-      <c r="H80" s="32"/>
-      <c r="I80" s="32"/>
-      <c r="J80" s="32"/>
-      <c r="K80" s="32"/>
-      <c r="L80" s="32"/>
-      <c r="M80" s="32"/>
-      <c r="O80" s="32" t="s">
+      <c r="C80" s="64"/>
+      <c r="D80" s="64"/>
+      <c r="E80" s="64"/>
+      <c r="F80" s="64"/>
+      <c r="G80" s="64"/>
+      <c r="H80" s="64"/>
+      <c r="I80" s="64"/>
+      <c r="J80" s="64"/>
+      <c r="K80" s="64"/>
+      <c r="L80" s="64"/>
+      <c r="M80" s="64"/>
+      <c r="O80" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="P80" s="32"/>
-      <c r="Q80" s="32"/>
-      <c r="R80" s="32"/>
-      <c r="S80" s="32"/>
-      <c r="T80" s="32"/>
-      <c r="U80" s="32"/>
-      <c r="V80" s="32"/>
-      <c r="W80" s="32"/>
-      <c r="X80" s="32"/>
-      <c r="Y80" s="32"/>
-      <c r="Z80" s="32"/>
+      <c r="P80" s="64"/>
+      <c r="Q80" s="64"/>
+      <c r="R80" s="64"/>
+      <c r="S80" s="64"/>
+      <c r="T80" s="64"/>
+      <c r="U80" s="64"/>
+      <c r="V80" s="64"/>
+      <c r="W80" s="64"/>
+      <c r="X80" s="64"/>
+      <c r="Y80" s="64"/>
+      <c r="Z80" s="64"/>
     </row>
     <row r="81" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B81" s="24" t="s">
@@ -4301,23 +4275,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B6:M6"/>
+    <mergeCell ref="O6:Z6"/>
+    <mergeCell ref="B8:M8"/>
+    <mergeCell ref="E9:M12"/>
+    <mergeCell ref="O8:Z8"/>
+    <mergeCell ref="R9:Z12"/>
+    <mergeCell ref="O13:Z13"/>
+    <mergeCell ref="B21:M21"/>
+    <mergeCell ref="O21:Z21"/>
+    <mergeCell ref="B33:M33"/>
+    <mergeCell ref="O33:Z33"/>
     <mergeCell ref="B49:M49"/>
     <mergeCell ref="O49:Z49"/>
     <mergeCell ref="B65:M65"/>
     <mergeCell ref="O65:Z65"/>
     <mergeCell ref="B80:M80"/>
     <mergeCell ref="O80:Z80"/>
-    <mergeCell ref="O13:Z13"/>
-    <mergeCell ref="B21:M21"/>
-    <mergeCell ref="O21:Z21"/>
-    <mergeCell ref="B33:M33"/>
-    <mergeCell ref="O33:Z33"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="O6:Z6"/>
-    <mergeCell ref="B8:M8"/>
-    <mergeCell ref="E9:M12"/>
-    <mergeCell ref="O8:Z8"/>
-    <mergeCell ref="R9:Z12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4326,9 +4300,83 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67740437-DAD4-467A-873C-E376A4EC5658}">
-  <dimension ref="A1"/>
+  <dimension ref="B6:T14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B6" s="71" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="71"/>
+      <c r="D6" s="71"/>
+      <c r="E6" s="71"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="71"/>
+      <c r="L6" s="71" t="s">
+        <v>24</v>
+      </c>
+      <c r="M6" s="71"/>
+      <c r="N6" s="71"/>
+      <c r="O6" s="71"/>
+      <c r="P6" s="71"/>
+      <c r="Q6" s="71"/>
+      <c r="R6" s="71"/>
+      <c r="S6" s="71"/>
+      <c r="T6" s="71"/>
+    </row>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8">
+        <f xml:space="preserve"> 100000</f>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="L6:T6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>